<commit_message>
ajoute le g7 de gestion MQTT
</commit_message>
<xml_diff>
--- a/G7.xlsx
+++ b/G7.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\devs\Detection voiture portail\BLE tag\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\devs\Detection voiture portail\BLE tag\SmartPortal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4386588C-5A59-476F-B4D9-E58EF20D2AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8624173A-F565-4307-B0F4-F39309C71AEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5685" yWindow="900" windowWidth="16410" windowHeight="11505" xr2:uid="{C1770F55-6E77-4222-A4D7-E888E4326736}"/>
+    <workbookView xWindow="5190" yWindow="915" windowWidth="16410" windowHeight="14250" activeTab="2" xr2:uid="{C1770F55-6E77-4222-A4D7-E888E4326736}"/>
   </bookViews>
   <sheets>
     <sheet name="Principal" sheetId="1" r:id="rId1"/>
     <sheet name="Reset" sheetId="3" r:id="rId2"/>
+    <sheet name="Commandes" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="37">
   <si>
     <t>Init</t>
   </si>
@@ -79,9 +80,6 @@
     <t>Bouton reset ?</t>
   </si>
   <si>
-    <t>+ 10 sec durée étape en cours (hors étapes 0, 11, 10)</t>
-  </si>
-  <si>
     <t>Réinit G7.Principal</t>
   </si>
   <si>
@@ -113,6 +111,33 @@
   </si>
   <si>
     <t>Autre (Echo 1 ou 2 pendant 2sec)</t>
+  </si>
+  <si>
+    <t>Les commandes sont transmisent via MQTT</t>
+  </si>
+  <si>
+    <t>+ 10 sec durée étape en cours (hors étapes P0, P11, P10)</t>
+  </si>
+  <si>
+    <t>CMD=CLOSE &amp; portail ouvert</t>
+  </si>
+  <si>
+    <t>CMD=OPEN &amp; portail fermé &amp; Hors étapes (P40)</t>
+  </si>
+  <si>
+    <t>Init (wifi et subscriber)</t>
+  </si>
+  <si>
+    <t>Activation Led orange</t>
+  </si>
+  <si>
+    <t>Attente 30 sec</t>
+  </si>
+  <si>
+    <t>Check MQTT</t>
+  </si>
+  <si>
+    <t>…</t>
   </si>
 </sst>
 </file>
@@ -196,7 +221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -223,6 +248,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -661,7 +689,7 @@
         <v>3</v>
       </c>
       <c r="P11" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -685,7 +713,7 @@
         <v>20</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="4:16" x14ac:dyDescent="0.25">
@@ -698,7 +726,7 @@
         <v>3</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -711,7 +739,7 @@
         <v>21</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="5:16" x14ac:dyDescent="0.25">
@@ -768,7 +796,7 @@
         <v>3</v>
       </c>
       <c r="P21" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -849,7 +877,7 @@
         <v>3</v>
       </c>
       <c r="P27" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -871,7 +899,7 @@
         <v>41</v>
       </c>
       <c r="P29" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="30" spans="5:16" x14ac:dyDescent="0.25">
@@ -887,13 +915,13 @@
         <v>3</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O31" s="1" t="s">
         <v>3</v>
       </c>
       <c r="P31" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="32" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -912,7 +940,7 @@
         <v>42</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O33" s="2" t="s">
         <v>2</v>
@@ -1081,7 +1109,7 @@
         <v>3</v>
       </c>
       <c r="P7" s="9" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="4:16" x14ac:dyDescent="0.25">
@@ -1137,7 +1165,7 @@
         <v>10</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="4:16" x14ac:dyDescent="0.25">
@@ -1158,6 +1186,306 @@
     </row>
     <row r="15" spans="4:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E15" s="5">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF81CEF6-863F-49BA-8D73-2C98F4EEFDFE}">
+  <dimension ref="D1:AC21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="50" width="3.7109375" style="1" customWidth="1"/>
+    <col min="51" max="16384" width="11.42578125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="4:29" x14ac:dyDescent="0.25">
+      <c r="E1" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="4:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" spans="4:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D3" s="4"/>
+      <c r="E3" s="5">
+        <v>0</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="4:29" x14ac:dyDescent="0.25">
+      <c r="E4" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="4:29" x14ac:dyDescent="0.25">
+      <c r="E5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="S5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="V5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="W5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="X5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="Z5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB5" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="4:29" x14ac:dyDescent="0.25">
+      <c r="E6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AB6" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="4:29" x14ac:dyDescent="0.25">
+      <c r="E7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="P7" s="9"/>
+      <c r="AB7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC7" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="4:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E8" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="AB8" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="4:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D9" s="4"/>
+      <c r="E9" s="5">
+        <v>1</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB9" s="5">
+        <v>11</v>
+      </c>
+      <c r="AC9" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="4:29" x14ac:dyDescent="0.25">
+      <c r="E10" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AB10" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="4:29" x14ac:dyDescent="0.25">
+      <c r="E11" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC11" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="4:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E12" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O12" s="2"/>
+      <c r="R12" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AB12" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="4:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="P13" s="9"/>
+      <c r="R13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="S13" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB13" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="4:29" x14ac:dyDescent="0.25">
+      <c r="E14" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O14" s="2"/>
+      <c r="R14" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="4:29" x14ac:dyDescent="0.25">
+      <c r="E15" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="R15" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="4:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E16" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="R16" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="5:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E17" s="5">
+        <v>10</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E18" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F18" s="6"/>
+    </row>
+    <row r="19" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E19" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="5:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E20" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="5:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E21" s="5">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
implémente les messages MQTT
</commit_message>
<xml_diff>
--- a/G7.xlsx
+++ b/G7.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\devs\Detection voiture portail\BLE tag\SmartPortal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8624173A-F565-4307-B0F4-F39309C71AEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E727630-DD45-4DA2-A03F-5E31B0C54C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5190" yWindow="915" windowWidth="16410" windowHeight="14250" activeTab="2" xr2:uid="{C1770F55-6E77-4222-A4D7-E888E4326736}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{C1770F55-6E77-4222-A4D7-E888E4326736}"/>
   </bookViews>
   <sheets>
     <sheet name="Principal" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="38">
   <si>
     <t>Init</t>
   </si>
@@ -122,9 +122,6 @@
     <t>CMD=CLOSE &amp; portail ouvert</t>
   </si>
   <si>
-    <t>CMD=OPEN &amp; portail fermé &amp; Hors étapes (P40)</t>
-  </si>
-  <si>
     <t>Init (wifi et subscriber)</t>
   </si>
   <si>
@@ -138,6 +135,12 @@
   </si>
   <si>
     <t>…</t>
+  </si>
+  <si>
+    <t>(bouton ouvrir | CMD=OPEN) &amp; portail fermé &amp; Hors étapes (P40)</t>
+  </si>
+  <si>
+    <t>portail fermé pendant 10sec</t>
   </si>
 </sst>
 </file>
@@ -1196,36 +1199,36 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF81CEF6-863F-49BA-8D73-2C98F4EEFDFE}">
-  <dimension ref="D1:AC21"/>
+  <dimension ref="D1:AH23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="50" width="3.7109375" style="1" customWidth="1"/>
     <col min="51" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="4:29" x14ac:dyDescent="0.25">
+    <row r="1" spans="4:34" x14ac:dyDescent="0.25">
       <c r="E1" s="10" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="4:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="4:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="4:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="4:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D3" s="4"/>
       <c r="E3" s="5">
         <v>0</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="4:29" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="4:34" x14ac:dyDescent="0.25">
       <c r="E4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="4:29" x14ac:dyDescent="0.25">
+    <row r="5" spans="4:34" x14ac:dyDescent="0.25">
       <c r="E5" s="2" t="s">
         <v>2</v>
       </c>
@@ -1296,18 +1299,33 @@
         <v>3</v>
       </c>
       <c r="AB5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG5" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="4:29" x14ac:dyDescent="0.25">
+    <row r="6" spans="4:34" x14ac:dyDescent="0.25">
       <c r="E6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="AB6" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="4:29" x14ac:dyDescent="0.25">
+      <c r="AG6" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="4:34" x14ac:dyDescent="0.25">
       <c r="E7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1315,149 +1333,169 @@
         <v>4</v>
       </c>
       <c r="P7" s="9"/>
-      <c r="AB7" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="AC7" s="6" t="s">
+      <c r="U7" s="9"/>
+      <c r="AG7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH7" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="4:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="4:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E8" s="2" t="s">
         <v>2</v>
       </c>
       <c r="O8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="AB8" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="4:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T8" s="2"/>
+      <c r="W8" s="2"/>
+      <c r="AG8" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="4:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D9" s="4"/>
       <c r="E9" s="5">
         <v>1</v>
       </c>
       <c r="F9" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="AG9" s="5">
+        <v>11</v>
+      </c>
+      <c r="AH9" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="4:34" x14ac:dyDescent="0.25">
+      <c r="E10" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG10" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="4:34" x14ac:dyDescent="0.25">
+      <c r="E11" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="S11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="T11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="U11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="V11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="W11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AG11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH11" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="4:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E12" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O12" s="2"/>
+      <c r="T12" s="2"/>
+      <c r="W12" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG12" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="4:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="P13" s="9"/>
+      <c r="U13" s="9"/>
+      <c r="W13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="X13" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="AG13" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="4:34" x14ac:dyDescent="0.25">
+      <c r="E14" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O14" s="2"/>
+      <c r="T14" s="2"/>
+      <c r="W14" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="4:34" x14ac:dyDescent="0.25">
+      <c r="E15" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="W15" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="4:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E16" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="W16" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="AB9" s="5">
-        <v>11</v>
-      </c>
-      <c r="AC9" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="4:29" x14ac:dyDescent="0.25">
-      <c r="E10" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="AB10" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="4:29" x14ac:dyDescent="0.25">
-      <c r="E11" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="N11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="O11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="P11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="R11" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AB11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="AC11" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="4:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E12" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="O12" s="2"/>
-      <c r="R12" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="AB12" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="4:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="P13" s="9"/>
-      <c r="R13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="S13" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB13" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="4:29" x14ac:dyDescent="0.25">
-      <c r="E14" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="O14" s="2"/>
-      <c r="R14" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="4:29" x14ac:dyDescent="0.25">
-      <c r="E15" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="R15" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="4:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E16" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="R16" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="17" spans="5:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1478,14 +1516,29 @@
       <c r="E19" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="20" spans="5:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F19" s="6"/>
+    </row>
+    <row r="20" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E20" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E21" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F21" s="6"/>
+    </row>
+    <row r="22" spans="5:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E22" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="5:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E21" s="5">
+    <row r="23" spans="5:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E23" s="5">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix le fonctionnement global
</commit_message>
<xml_diff>
--- a/G7.xlsx
+++ b/G7.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\devs\Detection voiture portail\BLE tag\SmartPortal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F691218-7462-4553-A593-AC4C96C844FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DAF2304-3F0C-4799-ACBD-978898B5D3DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{C1770F55-6E77-4222-A4D7-E888E4326736}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C1770F55-6E77-4222-A4D7-E888E4326736}"/>
   </bookViews>
   <sheets>
     <sheet name="Principal" sheetId="1" r:id="rId1"/>
@@ -113,9 +113,6 @@
     <t>Les commandes sont transmisent via MQTT</t>
   </si>
   <si>
-    <t>+ 10 sec durée étape en cours (hors étapes P0, P11, P10)</t>
-  </si>
-  <si>
     <t>Activation Led orange</t>
   </si>
   <si>
@@ -144,6 +141,9 @@
   </si>
   <si>
     <t>↑ Ouverture portail</t>
+  </si>
+  <si>
+    <t>+ 60 sec durée étape en cours (hors étapes P0, P11, P10)</t>
   </si>
 </sst>
 </file>
@@ -899,7 +899,7 @@
         <v>40</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O29" s="5">
         <v>41</v>
@@ -1115,7 +1115,7 @@
         <v>3</v>
       </c>
       <c r="P7" s="9" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="4:16" x14ac:dyDescent="0.25">
@@ -1223,7 +1223,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="4:52" x14ac:dyDescent="0.25">
@@ -1416,13 +1416,13 @@
         <v>1</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AY9" s="5">
         <v>11</v>
       </c>
       <c r="AZ9" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="4:52" x14ac:dyDescent="0.25">
@@ -1549,7 +1549,7 @@
         <v>3</v>
       </c>
       <c r="AZ11" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="4:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1573,7 +1573,7 @@
         <v>3</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="P13" s="9"/>
       <c r="U13" s="9"/>
@@ -1581,13 +1581,13 @@
         <v>3</v>
       </c>
       <c r="X13" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AO13" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AP13" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AY13" s="5">
         <v>0</v>
@@ -1622,10 +1622,10 @@
         <v>2</v>
       </c>
       <c r="W16" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="AO16" s="5">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="5:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1633,7 +1633,7 @@
         <v>10</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="5:6" x14ac:dyDescent="0.25">
@@ -1653,7 +1653,7 @@
         <v>3</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="5:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
modifie l'étape de detection tag et debug général pour tests
</commit_message>
<xml_diff>
--- a/G7.xlsx
+++ b/G7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\devs\Detection voiture portail\BLE tag\SmartPortal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DAF2304-3F0C-4799-ACBD-978898B5D3DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2804B1C1-0C94-49D4-AF86-AE3EDF197377}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C1770F55-6E77-4222-A4D7-E888E4326736}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="37">
   <si>
     <t>Init</t>
   </si>
@@ -86,18 +86,6 @@
     <t>Attente disparition badge et Portillon fermé</t>
   </si>
   <si>
-    <t>Fin lecture Badge</t>
-  </si>
-  <si>
-    <t>Début Lecture badge</t>
-  </si>
-  <si>
-    <t>Identification badge</t>
-  </si>
-  <si>
-    <t>Echec Identification</t>
-  </si>
-  <si>
     <t>Attente portail ouvert pendant 10sec</t>
   </si>
   <si>
@@ -144,6 +132,12 @@
   </si>
   <si>
     <t>+ 60 sec durée étape en cours (hors étapes P0, P11, P10)</t>
+  </si>
+  <si>
+    <t>Lecture badge</t>
+  </si>
+  <si>
+    <t>Echec Identification après 10 sec</t>
   </si>
 </sst>
 </file>
@@ -573,7 +567,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD5CF4F5-A8CE-4E84-A714-B5CF2F5A0A1F}">
-  <dimension ref="D2:P41"/>
+  <dimension ref="D2:P38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="50" width="3.7109375" style="1" customWidth="1"/>
@@ -719,7 +713,7 @@
         <v>20</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="4:16" x14ac:dyDescent="0.25">
@@ -728,305 +722,285 @@
       </c>
     </row>
     <row r="16" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E16" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F16" s="6" t="s">
+      <c r="E16" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="E17" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="E18" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P18" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E19" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E20" s="5">
+        <v>30</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="O20" s="5">
+        <v>10</v>
+      </c>
+      <c r="P20" s="7"/>
+    </row>
+    <row r="21" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="E21" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="E22" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O22" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="E23" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O23" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="E24" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P24" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E25" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O25" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E26" s="5">
+        <v>40</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="O26" s="5">
+        <v>41</v>
+      </c>
+      <c r="P26" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="E27" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O27" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="E28" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F28" s="6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="17" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E17" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E18" s="5">
-        <v>21</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="19" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E19" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M19" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="N19" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="O19" s="1" t="s">
+      <c r="O28" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="P28" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E29" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O29" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="P29" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E30" s="5">
+        <v>42</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="O30" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="E31" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="O31" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="E32" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N32" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O32" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E20" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="O20" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E21" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F21" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="O21" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="P21" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E22" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="O22" s="1" t="s">
+      <c r="P32" s="6"/>
+    </row>
+    <row r="33" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E33" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E34" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E35" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F35" s="6"/>
+    </row>
+    <row r="36" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E36" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="5:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E37" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E23" s="5">
-        <v>30</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="O23" s="5">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="24" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E24" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E25" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="L25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="N25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="O25" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E26" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="O26" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E27" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="O27" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="P27" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E28" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="O28" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E29" s="5">
-        <v>40</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="O29" s="5">
-        <v>41</v>
-      </c>
-      <c r="P29" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="30" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E30" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="O30" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="31" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E31" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="O31" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="P31" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="32" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E32" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="O32" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="P32" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="33" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E33" s="5">
-        <v>42</v>
-      </c>
-      <c r="F33" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="O33" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="34" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E34" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="O34" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="35" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E35" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I35" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="L35" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M35" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="N35" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="O35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P35" s="6"/>
-    </row>
-    <row r="36" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E36" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E37" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="38" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E38" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F38" s="6"/>
-    </row>
-    <row r="39" spans="5:16" x14ac:dyDescent="0.25">
-      <c r="E39" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="40" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E40" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="41" spans="5:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E41" s="5">
+    <row r="38" spans="5:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E38" s="5">
         <v>0</v>
       </c>
     </row>
@@ -1115,7 +1089,7 @@
         <v>3</v>
       </c>
       <c r="P7" s="9" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="4:16" x14ac:dyDescent="0.25">
@@ -1211,7 +1185,7 @@
   <sheetData>
     <row r="1" spans="4:52" x14ac:dyDescent="0.25">
       <c r="E1" s="10" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="4:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1223,7 +1197,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="4:52" x14ac:dyDescent="0.25">
@@ -1416,13 +1390,13 @@
         <v>1</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="AY9" s="5">
         <v>11</v>
       </c>
       <c r="AZ9" s="7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="4:52" x14ac:dyDescent="0.25">
@@ -1549,7 +1523,7 @@
         <v>3</v>
       </c>
       <c r="AZ11" s="6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="4:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1573,7 +1547,7 @@
         <v>3</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="P13" s="9"/>
       <c r="U13" s="9"/>
@@ -1581,13 +1555,13 @@
         <v>3</v>
       </c>
       <c r="X13" s="6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="AO13" s="1" t="s">
         <v>3</v>
       </c>
       <c r="AP13" s="6" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="AY13" s="5">
         <v>0</v>
@@ -1622,7 +1596,7 @@
         <v>2</v>
       </c>
       <c r="W16" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="AO16" s="5">
         <v>11</v>
@@ -1633,7 +1607,7 @@
         <v>10</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="5:6" x14ac:dyDescent="0.25">
@@ -1653,7 +1627,7 @@
         <v>3</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="5:6" x14ac:dyDescent="0.25">

</xml_diff>